<commit_message>
Actualiza base_datos.xlsx para centro Rancagua (San Fernando) con Detalle Comercial proyecto 19674586
Precios de instalación de cañerías Cu media/baja presión (1", 3/4", 1/2")
actualizados, y se agregan 3 ítems nuevos de conexiones y obras civiles
que no existían para el centro.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017De52GxAroFAQAPLWswWAQ
</commit_message>
<xml_diff>
--- a/base_datos.xlsx
+++ b/base_datos.xlsx
@@ -9559,7 +9559,7 @@
         </is>
       </c>
       <c r="H123" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="124">
@@ -10079,7 +10079,7 @@
         </is>
       </c>
       <c r="H136" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="137">
@@ -12159,7 +12159,7 @@
         </is>
       </c>
       <c r="H188" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="189">
@@ -18455,7 +18455,7 @@
         </is>
       </c>
       <c r="H123" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="124">
@@ -18975,7 +18975,7 @@
         </is>
       </c>
       <c r="H136" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="137">
@@ -21055,7 +21055,7 @@
         </is>
       </c>
       <c r="H188" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="189">
@@ -24195,7 +24195,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G258"/>
+  <dimension ref="A1:G260"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33228,6 +33228,76 @@
       </c>
       <c r="G258" t="n">
         <v>13480</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>INTERCONEX SERV. 2EST. AEREOS 4M3</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>1000086</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G259" t="n">
+        <v>95561</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>CONEXIÓN COCINA INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>1000036</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G260" t="n">
+        <v>23577</v>
       </c>
     </row>
   </sheetData>
@@ -33241,7 +33311,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G229"/>
+  <dimension ref="A1:G230"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -41259,6 +41329,41 @@
       </c>
       <c r="G229" t="n">
         <v>13000</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>METRO LINEAL DE REJA VERT. P/EST. AEREO</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>1000611</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G230" t="n">
+        <v>17338</v>
       </c>
     </row>
   </sheetData>

</xml_diff>